<commit_message>
Fix PCAP file accumulation - truncate between test cases
Critical fix: PCAP file was growing across test cases because we only cleared RunContext (in-memory) but not the actual file. Now truncating /data/network_capture.pcap in monitor container between test cases and resetting packet counter to 0.

Co-authored-by: bstHoang <139115555+bstHoang@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/batchstudent/Result/AnhDThe187386/OverallSummary.xlsx
+++ b/batchstudent/Result/AnhDThe187386/OverallSummary.xlsx
@@ -34,40 +34,37 @@
     <x:t>TC1</x:t>
   </x:si>
   <x:si>
-    <x:t>PASS</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
+    <x:t>FAIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Network flows: 2 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
   </x:si>
   <x:si>
     <x:t>TC2</x:t>
   </x:si>
   <x:si>
+    <x:t>Network flows: 3 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
+  </x:si>
+  <x:si>
     <x:t>TC3</x:t>
   </x:si>
   <x:si>
-    <x:t>FAIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Network flows: 3 FAIL (ALL-OR-NOTHING), 4 PASS</x:t>
+    <x:t>Network flows: 7 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
   </x:si>
   <x:si>
     <x:t>TC4</x:t>
   </x:si>
   <x:si>
-    <x:t>Network flows: 4 FAIL (ALL-OR-NOTHING), 7 PASS</x:t>
+    <x:t>Network flows: 11 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
   </x:si>
   <x:si>
     <x:t>TC5</x:t>
   </x:si>
   <x:si>
-    <x:t>Network flows: 2 FAIL (ALL-OR-NOTHING), 5 PASS</x:t>
-  </x:si>
-  <x:si>
     <x:t>TC6</x:t>
   </x:si>
   <x:si>
-    <x:t>Network flows: 9 FAIL (ALL-OR-NOTHING), 13 PASS</x:t>
+    <x:t>Network flows: 22 FAIL (ALL-OR-NOTHING), 0 PASS</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -468,7 +465,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C2" s="0">
-        <x:v>0.5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D2" s="0">
         <x:v>0.5</x:v>
@@ -485,21 +482,21 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="C3" s="0">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D3" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C4" s="0">
         <x:v>0</x:v>
@@ -516,7 +513,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C5" s="0">
         <x:v>0</x:v>
@@ -533,7 +530,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C6" s="0">
         <x:v>0</x:v>
@@ -542,15 +539,15 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:5">
       <x:c r="A7" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="0">
         <x:v>0</x:v>
@@ -559,7 +556,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>